<commit_message>
Updated cybersecurity requirements per taxonomy workbook (removed non-breaking spaces from text)
</commit_message>
<xml_diff>
--- a/distribution/reference_documents/working_material/cybersecurity requirements per taxonomy.xlsx
+++ b/distribution/reference_documents/working_material/cybersecurity requirements per taxonomy.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11210"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10511"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/charles.wilson/Documents/projects/AVCDL/source/reference_documents/working_material/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F00B508-F9A3-2843-9929-29C8F049B64B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BA179BA8-7143-034E-BCDA-9B497706832C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23420" yWindow="5500" windowWidth="23320" windowHeight="28160" xr2:uid="{56895247-3B3D-3147-A316-D5FB82A09ACE}"/>
+    <workbookView xWindow="27280" yWindow="3180" windowWidth="23320" windowHeight="28160" xr2:uid="{56895247-3B3D-3147-A316-D5FB82A09ACE}"/>
   </bookViews>
   <sheets>
-    <sheet name="layer-asset-property sort" sheetId="5" r:id="rId1"/>
+    <sheet name="cybersecurity requirements per " sheetId="5" r:id="rId1"/>
     <sheet name="asset-property-layer sort" sheetId="6" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
@@ -169,9 +169,6 @@
     <t>Logs shall be stored in a manner that protects the data's integrity.</t>
   </si>
   <si>
-    <t>The system shall enter a safe state when credentials are not available at time of use.</t>
-  </si>
-  <si>
     <t>Non-Repudiation</t>
   </si>
   <si>
@@ -187,9 +184,6 @@
     <t>Requirement</t>
   </si>
   <si>
-    <t>Logs shall avoid storing PII data and other regulated or sensitive data.</t>
-  </si>
-  <si>
     <t>Update payloads shall be encrypted at build time.</t>
   </si>
   <si>
@@ -223,9 +217,6 @@
     <t>Configuration data confidentiality shall be protected using access controls.</t>
   </si>
   <si>
-    <t>Configuration data shall only be accessed by authenticate entities.</t>
-  </si>
-  <si>
     <t>Configuration data authenticity shall be assured.</t>
   </si>
   <si>
@@ -268,9 +259,6 @@
     <t>Processes requiring human user authentication shall use authentication mechanisms (NIST SP 800-63).</t>
   </si>
   <si>
-    <t>Custom protocols shall use current best practices for authentication and key exchange (NIST SP 800-57,  63B, 131 and 133).</t>
-  </si>
-  <si>
     <t>Standard network protocols shall be secured using cybersecurity best practices.</t>
   </si>
   <si>
@@ -289,9 +277,6 @@
     <t>Communication crossing trust boundaries shall be authenticated.</t>
   </si>
   <si>
-    <t>Custom protocols that support a retry mechanism shall implement rate limiting.</t>
-  </si>
-  <si>
     <t>Persistent storage shall be encrypted.</t>
   </si>
   <si>
@@ -494,6 +479,21 @@
   </si>
   <si>
     <t>CR063</t>
+  </si>
+  <si>
+    <t>Configuration data shall only be accessed by authenticated entities.</t>
+  </si>
+  <si>
+    <t>The system shall enter a safe state when credentials are not available at time of use.</t>
+  </si>
+  <si>
+    <t>Logs shall avoid storing PII data and other regulated or sensitive data.</t>
+  </si>
+  <si>
+    <t>Custom protocols that support a retry mechanism shall implement rate limiting.</t>
+  </si>
+  <si>
+    <t>Custom protocols shall use current best practices for authentication and key exchange (NIST SP 800-57, 63B, 131 and 133).</t>
   </si>
 </sst>
 </file>
@@ -607,9 +607,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -647,7 +647,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -753,7 +753,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -895,7 +895,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -915,10 +915,10 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>0</v>
@@ -960,7 +960,7 @@
         <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>8</v>
@@ -975,13 +975,13 @@
         <v>4</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>12</v>
@@ -1016,14 +1016,14 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
@@ -1031,35 +1031,35 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T3" s="8"/>
       <c r="W3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -1067,23 +1067,23 @@
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T4" s="8"/>
       <c r="W4" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -1091,23 +1091,23 @@
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
       <c r="J5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T5" s="8"/>
       <c r="W5" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -1115,23 +1115,23 @@
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T6" s="8"/>
       <c r="W6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -1139,87 +1139,87 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T7" s="8"/>
       <c r="W7" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
       <c r="F8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T8" s="8"/>
       <c r="W8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T9" s="8"/>
       <c r="W9" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T10" s="8"/>
       <c r="W10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -1229,22 +1229,22 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N11" s="7"/>
       <c r="T11" s="8"/>
       <c r="W11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
         <v>24</v>
@@ -1254,43 +1254,43 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T12" s="8"/>
       <c r="W12" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H13" s="7"/>
       <c r="J13" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T13" s="8"/>
       <c r="W13" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -1300,20 +1300,20 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="H14" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T14" s="8"/>
       <c r="W14" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
         <v>35</v>
@@ -1323,20 +1323,20 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
       <c r="H15" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T15" s="8"/>
       <c r="W15" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -1348,19 +1348,19 @@
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T16" s="8"/>
       <c r="W16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -1372,19 +1372,19 @@
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T17" s="8"/>
       <c r="W17" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
@@ -1396,19 +1396,19 @@
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T18" s="8"/>
       <c r="W18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -1420,22 +1420,22 @@
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T19" s="8"/>
       <c r="W19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="7"/>
@@ -1444,22 +1444,22 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T20" s="8"/>
       <c r="W20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="7"/>
@@ -1467,19 +1467,19 @@
       <c r="F21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T21" s="8"/>
       <c r="W21" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -1487,7 +1487,7 @@
       <c r="C22" s="6"/>
       <c r="D22" s="7"/>
       <c r="E22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -1495,28 +1495,28 @@
       <c r="I22" s="7"/>
       <c r="J22" s="8"/>
       <c r="K22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T22" s="8"/>
       <c r="W22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
@@ -1526,23 +1526,23 @@
       <c r="I23" s="7"/>
       <c r="J23" s="8"/>
       <c r="K23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T23" s="8"/>
       <c r="W23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
@@ -1551,69 +1551,69 @@
       <c r="I24" s="7"/>
       <c r="J24" s="8"/>
       <c r="K24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T24" s="8"/>
       <c r="W24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>148</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
       <c r="G25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="8"/>
       <c r="K25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T25" s="8"/>
       <c r="W25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="8"/>
       <c r="K26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T26" s="8"/>
       <c r="W26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
@@ -1621,24 +1621,24 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="8"/>
       <c r="K27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T27" s="8"/>
       <c r="W27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
@@ -1647,26 +1647,26 @@
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T28" s="8"/>
       <c r="W28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
@@ -1676,44 +1676,44 @@
       <c r="I29" s="7"/>
       <c r="J29" s="8"/>
       <c r="L29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T29" s="8"/>
       <c r="W29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="8"/>
       <c r="L30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T30" s="8"/>
       <c r="W30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
         <v>20</v>
@@ -1725,23 +1725,23 @@
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J31" s="8"/>
       <c r="L31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T31" s="8"/>
       <c r="W31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
@@ -1749,24 +1749,24 @@
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I32" s="7"/>
       <c r="J32" s="8"/>
       <c r="M32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T32" s="8"/>
       <c r="W32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
@@ -1775,95 +1775,95 @@
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J33" s="8"/>
       <c r="M33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T33" s="8"/>
       <c r="W33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B34" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C34" s="6"/>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
       <c r="F34" s="7"/>
       <c r="G34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="7"/>
       <c r="J34" s="8"/>
       <c r="N34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T34" s="8"/>
       <c r="W34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B35" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
       <c r="G35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="8"/>
       <c r="N35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T35" s="8"/>
       <c r="W35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B36" t="s">
-        <v>44</v>
+        <v>149</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
       <c r="G36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="8"/>
       <c r="N36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T36" s="8"/>
       <c r="W36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B37" t="s">
         <v>31</v>
@@ -1874,21 +1874,21 @@
       <c r="F37" s="7"/>
       <c r="G37" s="7"/>
       <c r="H37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I37" s="7"/>
       <c r="J37" s="8"/>
       <c r="N37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T37" s="8"/>
       <c r="W37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B38" t="s">
         <v>32</v>
@@ -1899,21 +1899,21 @@
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="8"/>
       <c r="N38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T38" s="8"/>
       <c r="W38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B39" t="s">
         <v>11</v>
@@ -1925,26 +1925,26 @@
       <c r="G39" s="7"/>
       <c r="H39" s="7"/>
       <c r="I39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J39" s="8"/>
       <c r="N39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T39" s="8"/>
       <c r="W39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B40" t="s">
         <v>33</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D40" s="7"/>
       <c r="E40" s="7"/>
@@ -1954,25 +1954,25 @@
       <c r="I40" s="7"/>
       <c r="J40" s="8"/>
       <c r="O40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T40" s="8"/>
       <c r="W40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B41" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
@@ -1982,22 +1982,22 @@
       <c r="I41" s="7"/>
       <c r="J41" s="8"/>
       <c r="O41" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T41" s="8"/>
       <c r="W41" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B42" t="s">
         <v>41</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
@@ -2007,23 +2007,23 @@
       <c r="I42" s="7"/>
       <c r="J42" s="8"/>
       <c r="O42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T42" s="8"/>
       <c r="W42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B43" t="s">
         <v>43</v>
       </c>
       <c r="C43" s="6"/>
       <c r="D43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E43" s="7"/>
       <c r="F43" s="7"/>
@@ -2032,16 +2032,16 @@
       <c r="I43" s="7"/>
       <c r="J43" s="8"/>
       <c r="O43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T43" s="8"/>
       <c r="W43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B44" t="s">
         <v>22</v>
@@ -2049,7 +2049,7 @@
       <c r="C44" s="6"/>
       <c r="D44" s="7"/>
       <c r="E44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F44" s="7"/>
       <c r="G44" s="7"/>
@@ -2057,24 +2057,24 @@
       <c r="I44" s="7"/>
       <c r="J44" s="8"/>
       <c r="O44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T44" s="8"/>
       <c r="W44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B45" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C45" s="6"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F45" s="7"/>
       <c r="G45" s="7"/>
@@ -2082,16 +2082,16 @@
       <c r="I45" s="7"/>
       <c r="J45" s="8"/>
       <c r="O45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T45" s="8"/>
       <c r="W45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B46" t="s">
         <v>42</v>
@@ -2101,25 +2101,25 @@
       <c r="E46" s="7"/>
       <c r="F46" s="7"/>
       <c r="G46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H46" s="7"/>
       <c r="I46" s="7"/>
       <c r="J46" s="8"/>
       <c r="O46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T46" s="8"/>
       <c r="W46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B47" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C47" s="6"/>
       <c r="D47" s="7"/>
@@ -2127,27 +2127,27 @@
       <c r="F47" s="7"/>
       <c r="G47" s="7"/>
       <c r="H47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I47" s="7"/>
       <c r="J47" s="8"/>
       <c r="O47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T47" s="8"/>
       <c r="W47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B48" t="s">
         <v>30</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D48" s="7"/>
       <c r="E48" s="7"/>
@@ -2157,19 +2157,19 @@
       <c r="I48" s="7"/>
       <c r="J48" s="8"/>
       <c r="P48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T48" s="8"/>
       <c r="W48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B49" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C49" s="6"/>
       <c r="D49" s="7"/>
@@ -2177,27 +2177,27 @@
       <c r="F49" s="7"/>
       <c r="G49" s="7"/>
       <c r="H49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I49" s="7"/>
       <c r="J49" s="8"/>
       <c r="P49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T49" s="8"/>
       <c r="W49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B50" t="s">
         <v>28</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
@@ -2207,24 +2207,24 @@
       <c r="I50" s="7"/>
       <c r="J50" s="8"/>
       <c r="R50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S50" s="7"/>
       <c r="T50" s="8"/>
       <c r="W50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B51" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E51" s="7"/>
       <c r="F51" s="7"/>
@@ -2233,23 +2233,23 @@
       <c r="I51" s="7"/>
       <c r="J51" s="8"/>
       <c r="R51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S51" s="7"/>
       <c r="T51" s="8"/>
       <c r="W51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B52" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
@@ -2259,25 +2259,25 @@
       <c r="I52" s="7"/>
       <c r="J52" s="8"/>
       <c r="N52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T52" s="8"/>
       <c r="U52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B53" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
@@ -2287,25 +2287,25 @@
       <c r="I53" s="7"/>
       <c r="J53" s="8"/>
       <c r="P53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T53" s="8"/>
       <c r="U53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B54" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
@@ -2315,25 +2315,25 @@
       <c r="I54" s="7"/>
       <c r="J54" s="8"/>
       <c r="Q54" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T54" s="8"/>
       <c r="U54" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V54" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B55" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D55" s="7"/>
       <c r="E55" s="7"/>
@@ -2343,26 +2343,26 @@
       <c r="I55" s="7"/>
       <c r="J55" s="8"/>
       <c r="Q55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T55" s="8"/>
       <c r="U55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B56" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E56" s="7"/>
       <c r="F56" s="7"/>
@@ -2371,27 +2371,27 @@
       <c r="I56" s="7"/>
       <c r="J56" s="8"/>
       <c r="Q56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T56" s="8"/>
       <c r="U56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B57" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C57" s="6"/>
       <c r="D57" s="7"/>
       <c r="E57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F57" s="7"/>
       <c r="G57" s="7"/>
@@ -2399,102 +2399,102 @@
       <c r="I57" s="7"/>
       <c r="J57" s="8"/>
       <c r="Q57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T57" s="8"/>
       <c r="U57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B58" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C58" s="6"/>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
       <c r="G58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H58" s="7"/>
       <c r="I58" s="7"/>
       <c r="J58" s="8"/>
       <c r="Q58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T58" s="8"/>
       <c r="U58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B59" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="7"/>
       <c r="E59" s="7"/>
       <c r="F59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G59" s="7"/>
       <c r="H59" s="7"/>
       <c r="I59" s="7"/>
       <c r="J59" s="8"/>
       <c r="Q59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T59" s="8"/>
       <c r="V59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B60" t="s">
-        <v>77</v>
+        <v>152</v>
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
       <c r="F60" s="7"/>
       <c r="G60" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H60" s="7"/>
       <c r="I60" s="7"/>
       <c r="J60" s="8"/>
       <c r="Q60" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T60" s="8"/>
       <c r="V60" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B61" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D61" s="7"/>
       <c r="E61" s="7"/>
@@ -2504,22 +2504,22 @@
       <c r="I61" s="7"/>
       <c r="J61" s="8"/>
       <c r="Q61" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T61" s="8"/>
       <c r="U61" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B62" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D62" s="7"/>
       <c r="E62" s="7"/>
@@ -2529,15 +2529,15 @@
       <c r="I62" s="7"/>
       <c r="J62" s="8"/>
       <c r="S62" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T62" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B63" t="s">
         <v>36</v>
@@ -2545,7 +2545,7 @@
       <c r="C63" s="6"/>
       <c r="D63" s="7"/>
       <c r="E63" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="7"/>
@@ -2553,15 +2553,15 @@
       <c r="I63" s="7"/>
       <c r="J63" s="8"/>
       <c r="S63" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T63" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
@@ -2569,7 +2569,7 @@
       <c r="C64" s="6"/>
       <c r="D64" s="7"/>
       <c r="E64" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -2577,15 +2577,15 @@
       <c r="I64" s="7"/>
       <c r="J64" s="8"/>
       <c r="S64" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T64" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -2595,16 +2595,16 @@
       <c r="E65" s="7"/>
       <c r="F65" s="7"/>
       <c r="G65" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H65" s="7"/>
       <c r="I65" s="7"/>
       <c r="J65" s="8"/>
       <c r="S65" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T65" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>
@@ -2654,10 +2654,10 @@
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C1" s="9" t="s">
         <v>0</v>
@@ -2699,7 +2699,7 @@
         <v>23</v>
       </c>
       <c r="F2" s="5" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G2" s="5" t="s">
         <v>8</v>
@@ -2714,13 +2714,13 @@
         <v>4</v>
       </c>
       <c r="K2" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="L2" s="5" t="s">
         <v>3</v>
       </c>
       <c r="M2" s="5" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="N2" s="5" t="s">
         <v>12</v>
@@ -2755,14 +2755,14 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="C3" s="6"/>
       <c r="D3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="7"/>
@@ -2770,35 +2770,35 @@
       <c r="H3" s="7"/>
       <c r="I3" s="7"/>
       <c r="J3" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="O3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T3" s="8"/>
       <c r="W3" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B4" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C4" s="6"/>
       <c r="D4" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="7"/>
@@ -2806,23 +2806,23 @@
       <c r="H4" s="7"/>
       <c r="I4" s="7"/>
       <c r="J4" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T4" s="8"/>
       <c r="W4" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C5" s="6"/>
       <c r="D5" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E5" s="7"/>
       <c r="F5" s="7"/>
@@ -2830,23 +2830,23 @@
       <c r="H5" s="7"/>
       <c r="I5" s="7"/>
       <c r="J5" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T5" s="8"/>
       <c r="W5" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B6" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E6" s="7"/>
       <c r="F6" s="7"/>
@@ -2854,23 +2854,23 @@
       <c r="H6" s="7"/>
       <c r="I6" s="7"/>
       <c r="J6" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T6" s="8"/>
       <c r="W6" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C7" s="6"/>
       <c r="D7" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E7" s="7"/>
       <c r="F7" s="7"/>
@@ -2878,87 +2878,87 @@
       <c r="H7" s="7"/>
       <c r="I7" s="7"/>
       <c r="J7" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T7" s="8"/>
       <c r="W7" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B8" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C8" s="6"/>
       <c r="D8" s="7"/>
       <c r="E8" s="7"/>
       <c r="F8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G8" s="7"/>
       <c r="H8" s="7"/>
       <c r="I8" s="7"/>
       <c r="J8" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T8" s="8"/>
       <c r="W8" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B9" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C9" s="6"/>
       <c r="D9" s="7"/>
       <c r="E9" s="7"/>
       <c r="F9" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G9" s="7"/>
       <c r="H9" s="7"/>
       <c r="I9" s="7"/>
       <c r="J9" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T9" s="8"/>
       <c r="W9" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C10" s="6"/>
       <c r="D10" s="7"/>
       <c r="F10" s="7"/>
       <c r="G10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H10" s="7"/>
       <c r="I10" s="7"/>
       <c r="J10" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T10" s="8"/>
       <c r="W10" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B11" t="s">
         <v>7</v>
@@ -2968,22 +2968,22 @@
       <c r="E11" s="7"/>
       <c r="F11" s="7"/>
       <c r="G11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H11" s="7"/>
       <c r="I11" s="7"/>
       <c r="J11" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N11" s="7"/>
       <c r="T11" s="8"/>
       <c r="W11" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B12" t="s">
         <v>24</v>
@@ -2993,43 +2993,43 @@
       <c r="E12" s="7"/>
       <c r="F12" s="7"/>
       <c r="G12" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H12" s="7"/>
       <c r="I12" s="7"/>
       <c r="J12" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T12" s="8"/>
       <c r="W12" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B13" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C13" s="6"/>
       <c r="D13" s="7"/>
       <c r="F13" s="7"/>
       <c r="G13" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H13" s="7"/>
       <c r="J13" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T13" s="8"/>
       <c r="W13" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="14" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B14" t="s">
         <v>34</v>
@@ -3039,20 +3039,20 @@
       <c r="E14" s="7"/>
       <c r="F14" s="7"/>
       <c r="H14" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I14" s="7"/>
       <c r="J14" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T14" s="8"/>
       <c r="W14" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B15" t="s">
         <v>35</v>
@@ -3062,20 +3062,20 @@
       <c r="E15" s="7"/>
       <c r="F15" s="7"/>
       <c r="H15" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I15" s="7"/>
       <c r="J15" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T15" s="8"/>
       <c r="W15" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B16" t="s">
         <v>37</v>
@@ -3087,19 +3087,19 @@
       <c r="G16" s="7"/>
       <c r="H16" s="7"/>
       <c r="I16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J16" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T16" s="8"/>
       <c r="W16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B17" t="s">
         <v>38</v>
@@ -3111,19 +3111,19 @@
       <c r="G17" s="7"/>
       <c r="H17" s="7"/>
       <c r="I17" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J17" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T17" s="8"/>
       <c r="W17" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
         <v>25</v>
@@ -3135,19 +3135,19 @@
       <c r="G18" s="7"/>
       <c r="H18" s="7"/>
       <c r="I18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J18" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T18" s="8"/>
       <c r="W18" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="19" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B19" t="s">
         <v>26</v>
@@ -3159,22 +3159,22 @@
       <c r="G19" s="7"/>
       <c r="H19" s="7"/>
       <c r="I19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J19" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T19" s="8"/>
       <c r="W19" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="20" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B20" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="7"/>
@@ -3183,22 +3183,22 @@
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
       <c r="I20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J20" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T20" s="8"/>
       <c r="W20" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B21" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="7"/>
@@ -3206,19 +3206,19 @@
       <c r="F21" s="7"/>
       <c r="H21" s="7"/>
       <c r="I21" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J21" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T21" s="8"/>
       <c r="W21" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="22" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B22" t="s">
         <v>29</v>
@@ -3226,7 +3226,7 @@
       <c r="C22" s="6"/>
       <c r="D22" s="7"/>
       <c r="E22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -3234,28 +3234,28 @@
       <c r="I22" s="7"/>
       <c r="J22" s="8"/>
       <c r="K22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="L22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T22" s="8"/>
       <c r="W22" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B23" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D23" s="7"/>
       <c r="E23" s="7"/>
@@ -3265,23 +3265,23 @@
       <c r="I23" s="7"/>
       <c r="J23" s="8"/>
       <c r="K23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T23" s="8"/>
       <c r="W23" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="24" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B24" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E24" s="7"/>
       <c r="F24" s="7"/>
@@ -3290,69 +3290,69 @@
       <c r="I24" s="7"/>
       <c r="J24" s="8"/>
       <c r="K24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T24" s="8"/>
       <c r="W24" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="25" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B25" t="s">
-        <v>62</v>
+        <v>148</v>
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="7"/>
       <c r="E25" s="7"/>
       <c r="F25" s="7"/>
       <c r="G25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H25" s="7"/>
       <c r="I25" s="7"/>
       <c r="J25" s="8"/>
       <c r="K25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T25" s="8"/>
       <c r="W25" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="26" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B26" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="C26" s="6"/>
       <c r="D26" s="7"/>
       <c r="E26" s="7"/>
       <c r="F26" s="7"/>
       <c r="G26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H26" s="7"/>
       <c r="I26" s="7"/>
       <c r="J26" s="8"/>
       <c r="K26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T26" s="8"/>
       <c r="W26" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B27" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="C27" s="6"/>
       <c r="D27" s="7"/>
@@ -3360,24 +3360,24 @@
       <c r="F27" s="7"/>
       <c r="G27" s="7"/>
       <c r="H27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I27" s="7"/>
       <c r="J27" s="8"/>
       <c r="K27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T27" s="8"/>
       <c r="W27" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B28" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="C28" s="6"/>
       <c r="D28" s="7"/>
@@ -3386,26 +3386,26 @@
       <c r="G28" s="7"/>
       <c r="H28" s="7"/>
       <c r="I28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J28" s="8"/>
       <c r="K28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T28" s="8"/>
       <c r="W28" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="29" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B29" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D29" s="7"/>
       <c r="E29" s="7"/>
@@ -3415,44 +3415,44 @@
       <c r="I29" s="7"/>
       <c r="J29" s="8"/>
       <c r="L29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="N29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T29" s="8"/>
       <c r="W29" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B30" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C30" s="6"/>
       <c r="D30" s="7"/>
       <c r="E30" s="7"/>
       <c r="F30" s="7"/>
       <c r="G30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H30" s="7"/>
       <c r="I30" s="7"/>
       <c r="J30" s="8"/>
       <c r="L30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T30" s="8"/>
       <c r="W30" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B31" t="s">
         <v>20</v>
@@ -3464,23 +3464,23 @@
       <c r="G31" s="7"/>
       <c r="H31" s="7"/>
       <c r="I31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J31" s="8"/>
       <c r="L31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T31" s="8"/>
       <c r="W31" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="32" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B32" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="C32" s="6"/>
       <c r="D32" s="7"/>
@@ -3488,24 +3488,24 @@
       <c r="F32" s="7"/>
       <c r="G32" s="7"/>
       <c r="H32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I32" s="7"/>
       <c r="J32" s="8"/>
       <c r="M32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T32" s="8"/>
       <c r="W32" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="33" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B33" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="C33" s="6"/>
       <c r="D33" s="7"/>
@@ -3514,26 +3514,26 @@
       <c r="G33" s="7"/>
       <c r="H33" s="7"/>
       <c r="I33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J33" s="8"/>
       <c r="M33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T33" s="8"/>
       <c r="W33" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="34" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D34" s="7"/>
       <c r="E34" s="7"/>
@@ -3543,94 +3543,94 @@
       <c r="I34" s="7"/>
       <c r="J34" s="8"/>
       <c r="N34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T34" s="8"/>
       <c r="U34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V34" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="35" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B35" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="C35" s="6"/>
       <c r="D35" s="7"/>
       <c r="E35" s="7"/>
       <c r="F35" s="7"/>
       <c r="G35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="7"/>
       <c r="J35" s="8"/>
       <c r="N35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T35" s="8"/>
       <c r="W35" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="36" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B36" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C36" s="6"/>
       <c r="D36" s="7"/>
       <c r="E36" s="7"/>
       <c r="F36" s="7"/>
       <c r="G36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="7"/>
       <c r="J36" s="8"/>
       <c r="N36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T36" s="8"/>
       <c r="W36" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="37" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B37" t="s">
-        <v>44</v>
+        <v>149</v>
       </c>
       <c r="C37" s="6"/>
       <c r="D37" s="7"/>
       <c r="E37" s="7"/>
       <c r="F37" s="7"/>
       <c r="G37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="7"/>
       <c r="J37" s="8"/>
       <c r="N37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T37" s="8"/>
       <c r="W37" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="38" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B38" t="s">
         <v>31</v>
@@ -3641,21 +3641,21 @@
       <c r="F38" s="7"/>
       <c r="G38" s="7"/>
       <c r="H38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I38" s="7"/>
       <c r="J38" s="8"/>
       <c r="N38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T38" s="8"/>
       <c r="W38" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="39" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B39" t="s">
         <v>32</v>
@@ -3666,21 +3666,21 @@
       <c r="F39" s="7"/>
       <c r="G39" s="7"/>
       <c r="H39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I39" s="7"/>
       <c r="J39" s="8"/>
       <c r="N39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T39" s="8"/>
       <c r="W39" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B40" t="s">
         <v>11</v>
@@ -3692,26 +3692,26 @@
       <c r="G40" s="7"/>
       <c r="H40" s="7"/>
       <c r="I40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="J40" s="8"/>
       <c r="N40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T40" s="8"/>
       <c r="W40" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B41" t="s">
         <v>33</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D41" s="7"/>
       <c r="E41" s="7"/>
@@ -3721,22 +3721,22 @@
       <c r="I41" s="7"/>
       <c r="J41" s="8"/>
       <c r="O41" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T41" s="8"/>
       <c r="W41" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B42" t="s">
-        <v>50</v>
+        <v>150</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D42" s="7"/>
       <c r="E42" s="7"/>
@@ -3746,25 +3746,25 @@
       <c r="I42" s="7"/>
       <c r="J42" s="8"/>
       <c r="O42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T42" s="8"/>
       <c r="W42" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="43" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B43" t="s">
         <v>41</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D43" s="7"/>
       <c r="E43" s="7"/>
@@ -3774,23 +3774,23 @@
       <c r="I43" s="7"/>
       <c r="J43" s="8"/>
       <c r="O43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T43" s="8"/>
       <c r="W43" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="44" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B44" t="s">
         <v>43</v>
       </c>
       <c r="C44" s="6"/>
       <c r="D44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E44" s="7"/>
       <c r="F44" s="7"/>
@@ -3799,16 +3799,16 @@
       <c r="I44" s="7"/>
       <c r="J44" s="8"/>
       <c r="O44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T44" s="8"/>
       <c r="W44" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="45" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B45" t="s">
         <v>22</v>
@@ -3816,7 +3816,7 @@
       <c r="C45" s="6"/>
       <c r="D45" s="7"/>
       <c r="E45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F45" s="7"/>
       <c r="G45" s="7"/>
@@ -3824,24 +3824,24 @@
       <c r="I45" s="7"/>
       <c r="J45" s="8"/>
       <c r="O45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T45" s="8"/>
       <c r="W45" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="46" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B46" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="C46" s="6"/>
       <c r="D46" s="7"/>
       <c r="E46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F46" s="7"/>
       <c r="G46" s="7"/>
@@ -3849,16 +3849,16 @@
       <c r="I46" s="7"/>
       <c r="J46" s="8"/>
       <c r="O46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T46" s="8"/>
       <c r="W46" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B47" t="s">
         <v>42</v>
@@ -3868,25 +3868,25 @@
       <c r="E47" s="7"/>
       <c r="F47" s="7"/>
       <c r="G47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H47" s="7"/>
       <c r="I47" s="7"/>
       <c r="J47" s="8"/>
       <c r="O47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T47" s="8"/>
       <c r="W47" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="48" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B48" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="C48" s="6"/>
       <c r="D48" s="7"/>
@@ -3894,27 +3894,27 @@
       <c r="F48" s="7"/>
       <c r="G48" s="7"/>
       <c r="H48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I48" s="7"/>
       <c r="J48" s="8"/>
       <c r="O48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T48" s="8"/>
       <c r="W48" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="49" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B49" t="s">
         <v>30</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D49" s="7"/>
       <c r="E49" s="7"/>
@@ -3924,22 +3924,22 @@
       <c r="I49" s="7"/>
       <c r="J49" s="8"/>
       <c r="P49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T49" s="8"/>
       <c r="W49" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="50" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B50" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D50" s="7"/>
       <c r="E50" s="7"/>
@@ -3949,22 +3949,22 @@
       <c r="I50" s="7"/>
       <c r="J50" s="8"/>
       <c r="P50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T50" s="8"/>
       <c r="U50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V50" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="51" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B51" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="C51" s="6"/>
       <c r="D51" s="7"/>
@@ -3972,27 +3972,27 @@
       <c r="F51" s="7"/>
       <c r="G51" s="7"/>
       <c r="H51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="I51" s="7"/>
       <c r="J51" s="8"/>
       <c r="P51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T51" s="8"/>
       <c r="W51" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="52" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B52" t="s">
-        <v>79</v>
+        <v>75</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D52" s="7"/>
       <c r="E52" s="7"/>
@@ -4002,25 +4002,25 @@
       <c r="I52" s="7"/>
       <c r="J52" s="8"/>
       <c r="Q52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T52" s="8"/>
       <c r="U52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V52" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="53" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B53" t="s">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D53" s="7"/>
       <c r="E53" s="7"/>
@@ -4030,25 +4030,25 @@
       <c r="I53" s="7"/>
       <c r="J53" s="8"/>
       <c r="Q53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T53" s="8"/>
       <c r="U53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V53" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="54" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B54" t="s">
-        <v>78</v>
+        <v>74</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D54" s="7"/>
       <c r="E54" s="7"/>
@@ -4058,23 +4058,23 @@
       <c r="I54" s="7"/>
       <c r="J54" s="8"/>
       <c r="Q54" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T54" s="8"/>
       <c r="U54" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="55" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B55" t="s">
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="C55" s="6"/>
       <c r="D55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E55" s="7"/>
       <c r="F55" s="7"/>
@@ -4083,27 +4083,27 @@
       <c r="I55" s="7"/>
       <c r="J55" s="8"/>
       <c r="Q55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T55" s="8"/>
       <c r="U55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V55" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="56" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B56" t="s">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="C56" s="6"/>
       <c r="D56" s="7"/>
       <c r="E56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F56" s="7"/>
       <c r="G56" s="7"/>
@@ -4111,102 +4111,102 @@
       <c r="I56" s="7"/>
       <c r="J56" s="8"/>
       <c r="Q56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T56" s="8"/>
       <c r="U56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V56" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="57" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B57" t="s">
-        <v>84</v>
+        <v>151</v>
       </c>
       <c r="C57" s="6"/>
       <c r="D57" s="7"/>
       <c r="E57" s="7"/>
       <c r="F57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G57" s="7"/>
       <c r="H57" s="7"/>
       <c r="I57" s="7"/>
       <c r="J57" s="8"/>
       <c r="Q57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T57" s="8"/>
       <c r="V57" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="58" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B58" t="s">
-        <v>83</v>
+        <v>79</v>
       </c>
       <c r="C58" s="6"/>
       <c r="E58" s="7"/>
       <c r="F58" s="7"/>
       <c r="G58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H58" s="7"/>
       <c r="I58" s="7"/>
       <c r="J58" s="8"/>
       <c r="Q58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T58" s="8"/>
       <c r="U58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="V58" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="59" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B59" t="s">
-        <v>77</v>
+        <v>152</v>
       </c>
       <c r="C59" s="6"/>
       <c r="D59" s="7"/>
       <c r="E59" s="7"/>
       <c r="F59" s="7"/>
       <c r="G59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H59" s="7"/>
       <c r="I59" s="7"/>
       <c r="J59" s="8"/>
       <c r="Q59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T59" s="8"/>
       <c r="V59" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="60" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B60" t="s">
         <v>28</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D60" s="7"/>
       <c r="E60" s="7"/>
@@ -4216,24 +4216,24 @@
       <c r="I60" s="7"/>
       <c r="J60" s="8"/>
       <c r="R60" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S60" s="7"/>
       <c r="T60" s="8"/>
       <c r="W60" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="61" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B61" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="C61" s="6"/>
       <c r="D61" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E61" s="7"/>
       <c r="F61" s="7"/>
@@ -4242,23 +4242,23 @@
       <c r="I61" s="7"/>
       <c r="J61" s="8"/>
       <c r="R61" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="S61" s="7"/>
       <c r="T61" s="8"/>
       <c r="W61" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="62" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B62" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D62" s="7"/>
       <c r="E62" s="7"/>
@@ -4268,15 +4268,15 @@
       <c r="I62" s="7"/>
       <c r="J62" s="8"/>
       <c r="S62" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T62" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="63" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B63" t="s">
         <v>36</v>
@@ -4284,7 +4284,7 @@
       <c r="C63" s="6"/>
       <c r="D63" s="7"/>
       <c r="E63" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F63" s="7"/>
       <c r="G63" s="7"/>
@@ -4292,15 +4292,15 @@
       <c r="I63" s="7"/>
       <c r="J63" s="8"/>
       <c r="S63" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T63" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="64" spans="1:23" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B64" t="s">
         <v>39</v>
@@ -4308,7 +4308,7 @@
       <c r="C64" s="6"/>
       <c r="D64" s="7"/>
       <c r="E64" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F64" s="7"/>
       <c r="G64" s="7"/>
@@ -4316,15 +4316,15 @@
       <c r="I64" s="7"/>
       <c r="J64" s="8"/>
       <c r="S64" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T64" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="65" spans="1:20" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B65" t="s">
         <v>15</v>
@@ -4334,16 +4334,16 @@
       <c r="E65" s="7"/>
       <c r="F65" s="7"/>
       <c r="G65" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="H65" s="7"/>
       <c r="I65" s="7"/>
       <c r="J65" s="8"/>
       <c r="S65" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="T65" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
   </sheetData>

</xml_diff>